<commit_message>
fix(roadmap): correct batch count and timeline to hit 31 Aug 2026
- Batches: 33 -> 31 (based on 309 active repos, not 327 total)
- Timeline: 22 weeks -> 7 weeks (14 Jul - 31 Aug 2026)
- Dates now day-based offsets (not weeks)
- Phase 5 AB AppDev runs 2 batches/day to fit timeline
- Batch 31 correctly ends at Repos 307-309 (final 3, not 10)
</commit_message>
<xml_diff>
--- a/Documents/ADO to GitHub Migration Roadmap Abank.xlsx
+++ b/Documents/ADO to GitHub Migration Roadmap Abank.xlsx
@@ -493,7 +493,7 @@
   <dimension ref="B2:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -560,12 +560,12 @@
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Active Repos</t>
+          <t>Active Repos (to migrate)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>309 (excl. 18 empty repos)</t>
+          <t>309 (excl. 18 empty repos - confirmed skip)</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>33 batches (327 / 10, rounded up)</t>
+          <t>31 batches (309 active repos / 10, rounded up)</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>~22 weeks</t>
+          <t>~7 weeks</t>
         </is>
       </c>
     </row>
@@ -676,18 +676,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J52"/>
+  <dimension ref="B2:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="49" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
@@ -753,7 +753,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Align stakeholders on migration scope, approach (git mirror), timeline, and decision owners. Get sign-off on: master-&gt;main rename, empty repo disposition, collision rename, PR history acceptance.</t>
+          <t>Align stakeholders on migration scope, approach (git mirror), timeline, and decision owners. Get sign-off on: master-&gt;main rename, 18 empty repos disposition, 3 collision renames, PR history acceptance.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Provision GitHub Enterprise Cloud org (zeb-ai or abank). Configure Entra SSO + SCIM. Create org-level settings: default branch = main, secret scanning on, push protection on.</t>
+          <t>Provision GitHub Enterprise Cloud org. Configure Entra SSO + SCIM. Set org defaults: default branch = main, secret scanning on, push protection on.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>19 Jul 2026</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>16 Jul 2026</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Review extracted inventory (327 repos). Identify and confirm: 18 empty repos (skip/migrate), 3 collision renames, stale single-repo projects, wave groupings.</t>
+          <t>Review extracted inventory (309 active repos). Confirm: 18 empty repos skip, 3 collision renames, batch groupings by project and activity.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>19 Jul 2026</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Finalized Repo Inventory sheet with wave assignments</t>
+          <t>Finalized Repo Inventory with batch assignments</t>
         </is>
       </c>
     </row>
@@ -928,12 +928,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Script Development - Mirror</t>
+          <t>Script Dev - Mirror</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Develop git_mirror_migrate.py: iterates repo list, runs git clone --mirror from abdevopsdev and git push --mirror to GitHub. Supports dry-run mode, retry on failure, progress log, resume from last completed repo.</t>
+          <t>Develop git_mirror_migrate.py: git clone --mirror from abdevopsdev + git push --mirror to GitHub. Dry-run, retry, resume, master-&gt;main rename flag, per-repo progress log.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Script Development - Topics</t>
+          <t>Script Dev - Topics &amp; Teams</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Develop apply_topics_teams.py: reads workbook Target Topics + Target Team(s) columns, calls gh api to set topics and team permissions per repo. Dry-run mode.</t>
+          <t>Develop apply_topics_teams.py: read Target Topics + Teams from workbook, call gh api to set topics and repo permissions. Dry-run mode, idempotent.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1018,12 +1018,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Script Development - Ruleset</t>
+          <t>Script Dev - Rulesets</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Develop apply_rulesets.py: creates 3-4 Ruleset JSON templates (default-protect, require-review, file-size, comment-required), attaches to repos by topic. Dry-run mode.</t>
+          <t>Develop apply_rulesets.py: author 3-4 Ruleset JSON templates (default-protect, require-review, file-size, comment-required). Attach to repos by topic. Dry-run mode.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>apply_rulesets.py + ruleset JSON templates in github-config/</t>
+          <t>apply_rulesets.py + ruleset JSON templates</t>
         </is>
       </c>
     </row>
@@ -1063,12 +1063,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Script Development - Verify</t>
+          <t>Script Dev - Verify</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Develop post_migration_verify.py: for each migrated repo checks branch count, tag count, default branch, topics applied, team access, Ruleset attached. Outputs pass/fail per repo.</t>
+          <t>Develop post_migration_verify.py: per-repo checks (branch count, tag count, default branch, topics, team access, Ruleset). Pass/fail output per repo.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Test all four scripts against zeb-ai sandbox org (already on GitHub). Validate dry-run, retry, resume, error handling. Fix any issues before pilot.</t>
+          <t>Test all scripts against zeb-ai sandbox org. Validate dry-run, retry, resume, error handling. Fix issues before pilot.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Pilot - Batch 0 (2 repos)</t>
+          <t>Pilot - 2 repos</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Select 2 low-risk repos (1 from ScriptRefactoring + 1 small single-repo project). Run full end-to-end: mirror -&gt; topics -&gt; Ruleset -&gt; verify. Validate with repo owner. Retro findings fed back into scripts.</t>
+          <t>Select 2 low-risk repos (1 from ScriptRefactoring + 1 single-repo stale project). Run full end-to-end: mirror -&gt; topics -&gt; Ruleset -&gt; verify. Validate with repo owner.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1168,12 +1168,12 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Review pilot output: any missing branches/tags, topic errors, Ruleset attach failures, team permission issues. Fix scripts. Update runbook.</t>
+          <t>Review pilot output. Fix any branch/tag gaps, topic errors, Ruleset failures. Update runbook. Get sign-off to proceed.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Updated scripts, updated runbook</t>
+          <t>Updated scripts + runbook, sign-off to proceed</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Single-repo stale projects (last commit &gt; 2 years). Freeze ADO, mirror, apply topics + teams + Ruleset, verify, archive ADO repos. Notify owners.</t>
+          <t>Single-repo stale projects (last commit &gt; 2 yrs). Freeze ADO -&gt; mirror -&gt; topics + teams + Ruleset -&gt; verify -&gt; archive ADO. 24h freeze notice.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1258,12 +1258,12 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>01 Aug 2026</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Continue single-repo projects (moderately stale, 1-2 years). Same process: freeze -&gt; mirror -&gt; topics/teams/Ruleset -&gt; verify -&gt; archive.</t>
+          <t>Single-repo projects (1-2 yrs idle). Same process.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>01 Aug 2026</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>SSIS ETL project (5 repos) + remaining single-repo projects. Same cutover process.</t>
+          <t>SSIS ETL (5 repos) + remaining single-repo projects. Same process.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1348,12 +1348,12 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>15 Sep 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Non Binary (2 repos) + active single-repo projects (last commit &lt; 1 year). Increase freeze notice to 48h.</t>
+          <t>Non Binary (2) + active single-repo projects. 48h freeze notice.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1393,12 +1393,12 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>15 Sep 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>22 Sep 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>22 Sep 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>29 Sep 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>ScriptRefactoring project begins. 10 repos from SR. Freeze -&gt; mirror -&gt; topics (project-scriptrefactoring) -&gt; Ruleset -&gt; verify -&gt; archive.</t>
+          <t>ScriptRefactoring begins. First 10 SR repos. 48h freeze notice.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>29 Sep 2026</t>
+          <t>07 Aug 2026</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>06 Oct 2026</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1528,12 +1528,12 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>06 Oct 2026</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>13 Oct 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>13 Oct 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1618,12 +1618,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>27 Oct 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>ScriptRefactoring: final 16 repos. SR project fully migrated.</t>
+          <t>ScriptRefactoring: final 16 repos. SR fully migrated.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>27 Oct 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>AB AppDev begins. First 10 repos (low-traffic, oldest last-commit). Freeze -&gt; mirror -&gt; topics (project-ab-appdev) -&gt; verify -&gt; archive.</t>
+          <t>AB AppDev begins. First 10 repos (oldest last-commit). 48h freeze notice.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1708,12 +1708,12 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1843,12 +1843,12 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -1933,12 +1933,12 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -1978,12 +1978,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -2023,12 +2023,12 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2113,12 +2113,12 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2203,12 +2203,12 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2293,12 +2293,12 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2338,12 +2338,12 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2383,12 +2383,12 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2518,12 +2518,12 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2563,12 +2563,12 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2593,12 +2593,12 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Batch 31 (Repos 307-316)</t>
+          <t>Batch 31 (Repos 307-309)</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>AB AppDev: next 10 repos.</t>
+          <t>AB AppDev: final 3 repos. All 309 active repos migrated.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -2608,12 +2608,12 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -2623,97 +2623,97 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>10 AB AppDev repos on GitHub</t>
+          <t>All AB AppDev repos on GitHub</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="4" t="n">
+      <c r="B45" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Batch 32 (Repos 317-326)</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev: next 10 repos.</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Full Org Audit</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Run post_migration_verify.py across all 309 migrated repos. Every repo must have project-* topic, correct default branch, Ruleset attached, correct team access.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>08 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>27 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>29 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>10 AB AppDev repos on GitHub</t>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Audit report - all repos green</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="4" t="n">
+      <c r="B46" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Batch 33 (Repo 327)</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev: final repo. AB AppDev project fully migrated.</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>08 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Security Review</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Confirm: no repo public unintentionally, secret scanning enabled org-wide, push protection on, no hardcoded secrets flagged.</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>27 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>29 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>All 244 AB AppDev repos on GitHub</t>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Security sign-off</t>
         </is>
       </c>
     </row>
@@ -2728,127 +2728,127 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Full Org Audit</t>
+          <t>Consumer Redirect</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Run post_migration_verify.py across all 327 repos. Check: every repo has project-* topic, correct default branch, Ruleset attached, correct team access. Fix any gaps.</t>
+          <t>Update submodule URLs, CI/CD clone URLs, package feed refs, README badges pointing to abdevopsdev. Raise PRs per affected repo.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
+          <t>Team Leads</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>27 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>All consumers redirected to GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Phase 7</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>ADO Server Archive</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Set all migrated ADO repos to read-only. Communicate: ADO is archive-only. Retain 90 days as reference.</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Platform Team</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>31 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>ADO repos read-only, comms sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Phase 7</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Runbook Handover</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Deliver runbook to platform team (add repo, apply topics, request access, change Ruleset). Conduct 1h handover session.</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>22 Dec 2026</t>
-        </is>
-      </c>
-      <c r="I47" s="5" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>31 Aug 2026</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J47" s="5" t="inlineStr">
-        <is>
-          <t>Audit report - all repos green</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="5" t="n">
-        <v>46</v>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Security Review</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Confirm: no repo left public unintentionally, secret scanning enabled org-wide, push protection enabled, no hardcoded secrets in migrated repos (GitHub secret scan alert review).</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>22 Dec 2026</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr">
-        <is>
-          <t>Security sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="5" t="n">
-        <v>47</v>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Consumer Redirect</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Update all consumer references pointing to abdevopsdev: submodule URLs, CI/CD pipeline clone URLs, package feed references, README badges. Raise PRs per affected repo.</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>Team Leads</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>29 Dec 2026</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>All consumers redirected to GitHub</t>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>Runbook doc + handover session</t>
         </is>
       </c>
     </row>
@@ -2863,27 +2863,27 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>ADO Server Archive</t>
+          <t>ADO Decommission Planning</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Set all migrated ADO repos to read-only (disable push). Communicate to all teams: ADO is now archive-only. Retain for 90 days as reference.</t>
+          <t>Plan final ADO Server decommission 90 days post-archive. Confirm retention policy with Abank. Schedule infra team.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>Platform Team</t>
+          <t>Abank Infra</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>29 Dec 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>29 Dec 2026</t>
+          <t>31 Aug 2026</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -2892,96 +2892,6 @@
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>ADO repos read-only, comms sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>Phase 7</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>Runbook Handover</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>Deliver operational runbook to platform team: how to add new repos, apply topics, request team access, raise Ruleset changes. Conduct handover session.</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>29 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>05 Jan 2027</t>
-        </is>
-      </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>Runbook doc + handover session</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>Phase 7</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>ADO Decommission Planning</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>Plan final ADO Server decommission (90 days post archive). Confirm data retention policy with Abank. Schedule infra team for server removal.</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>Abank Infra</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>29 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>12 Jan 2027</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>Decommission plan signed off</t>
         </is>
@@ -2998,14 +2908,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H36"/>
+  <dimension ref="B2:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="56" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -3065,22 +2975,22 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>1 from ScriptRefactoring + 1 small single-repo project</t>
+          <t>1 ScriptRefactoring + 1 single-repo stale</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>End-to-end process validation</t>
+          <t>End-to-end validation</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -3102,22 +3012,22 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Single-repo stale projects (&gt;2 yrs idle)</t>
+          <t>Single-repo stale (&gt;2 yrs idle)</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Low risk warm-up</t>
+          <t>Low risk</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>25 Aug 2026</t>
+          <t>31 Jul 2026</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>01 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3049,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Single-repo projects (1-2 yrs idle)</t>
+          <t>Single-repo (1-2 yrs idle)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -3149,12 +3059,12 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>01 Aug 2026</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3176,22 +3086,22 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>SSIS ETL (5) + remaining single-repo projects</t>
+          <t>SSIS ETL (5) + single-repo projects</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Low-medium risk</t>
+          <t>Low-medium</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>08 Sep 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>15 Sep 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3213,22 +3123,22 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Non Binary (2) + active single-repo projects</t>
+          <t>Non Binary (2) + active single-repo</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Medium risk, 48h freeze</t>
+          <t>Medium, 48h freeze</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>15 Sep 2026</t>
+          <t>03 Aug 2026</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>22 Sep 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3255,17 +3165,17 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Medium risk</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>22 Sep 2026</t>
+          <t>04 Aug 2026</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>29 Sep 2026</t>
+          <t>05 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3292,17 +3202,17 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Medium risk</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>29 Sep 2026</t>
+          <t>07 Aug 2026</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>06 Oct 2026</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3329,17 +3239,17 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Medium risk</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>06 Oct 2026</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>13 Oct 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3366,17 +3276,17 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Medium risk</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>13 Oct 2026</t>
+          <t>09 Aug 2026</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3403,17 +3313,17 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Medium risk</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>10 Aug 2026</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>27 Oct 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3445,12 +3355,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>27 Oct 2026</t>
+          <t>11 Aug 2026</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3472,22 +3382,22 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>AB AppDev: first 10 (oldest last-commit)</t>
+          <t>AB AppDev: first 10 (oldest)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Higher risk, 48h freeze</t>
+          <t>Higher, 48h freeze</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>14 Aug 2026</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3514,17 +3424,17 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>15 Aug 2026</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3551,17 +3461,17 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>16 Aug 2026</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3588,17 +3498,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>10 Nov 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3625,17 +3535,17 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>18 Aug 2026</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3662,17 +3572,17 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>19 Aug 2026</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3699,17 +3609,17 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>20 Aug 2026</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3736,17 +3646,17 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>24 Nov 2026</t>
+          <t>21 Aug 2026</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3773,17 +3683,17 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>22 Aug 2026</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3810,17 +3720,17 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>01 Dec 2026</t>
+          <t>23 Aug 2026</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3847,17 +3757,17 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>24 Aug 2026</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3884,17 +3794,17 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3921,17 +3831,17 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3958,17 +3868,17 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>26 Aug 2026</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -3995,17 +3905,17 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4032,17 +3942,17 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>27 Aug 2026</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4069,17 +3979,17 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4106,17 +4016,17 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>28 Aug 2026</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4143,17 +4053,17 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4180,17 +4090,17 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>Higher</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4207,101 +4117,27 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Repos 307-316</t>
+          <t>Repos 307-309</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>AB AppDev: next 10</t>
+          <t>AB AppDev: final 3 repos</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Higher risk</t>
+          <t>All 309 repos migrated</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>08 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Batch 32</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Repos 317-326</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev: next 10</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Higher risk</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>08 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Batch 33</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Phase 5</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Repo 327</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev: final repo</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>AB AppDev fully migrated</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>08 Dec 2026</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>15 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -4370,7 +4206,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>309 repos are on `master`. GitHub default is `main`. Do we rename during migration or keep `master`?</t>
+          <t>309 repos are on `master`. GitHub default is `main`. Rename during migration or keep `master`?</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4380,12 +4216,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Rename to `main` during mirror step (recommended) OR keep `master` and set GitHub default branch to `master`</t>
+          <t>Rename to `main` during mirror step (recommended) OR keep `master` and set GitHub default to `master`</t>
         </is>
       </c>
     </row>
@@ -4410,7 +4246,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -4440,12 +4276,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Suffix the less-active copy (e.g. BAM-standalone) OR prefix with project (e.g. ab-appdev-BAM)</t>
+          <t>Suffix the less-active copy (e.g. BAM-standalone) OR prefix with project name</t>
         </is>
       </c>
     </row>
@@ -4470,12 +4306,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Accept loss + keep ADO read-only 90 days (recommended) OR engage GitHub PS for custom exporter (2-3 wks extra)</t>
+          <t>Accept loss + keep ADO read-only 90 days (recommended) OR engage GitHub PS for custom exporter</t>
         </is>
       </c>
     </row>
@@ -4500,12 +4336,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>21 Jul 2026</t>
+          <t>19 Jul 2026</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Apply default-protect Ruleset to all repos (recommended) OR migrate as-is with no protection</t>
+          <t>Apply default-protect Ruleset to all repos (recommended) OR migrate as-is</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4366,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>14 Jul 2026</t>
+          <t>17 Jul 2026</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4560,7 +4396,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>29 Dec 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4666,7 +4502,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -4706,7 +4542,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -4746,7 +4582,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -4781,12 +4617,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>28 Jul 2026</t>
+          <t>23 Jul 2026</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>04 Aug 2026</t>
+          <t>26 Jul 2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -4821,12 +4657,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>11 Aug 2026</t>
+          <t>28 Jul 2026</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>18 Aug 2026</t>
+          <t>29 Jul 2026</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">

</xml_diff>